<commit_message>
Barkod kutije (package_barcode): skeniranje kutije dodaje pieces_per_package komada
Backend: Product.package_barcode (unique po klijentu zajedno sa barcode,
zahteva pieces_per_package > 0), by-barcode vraca scan_unit/scan_qty,
POST /products/{id}/barcode i /products/quick primaju vrstu barkoda,
Excel uvoz kolona 'Barkod kutije'. Mobilna: Prijem/Popis dodaju celu kutiju,
izbor komad/kutija za nepoznat barkod, polje u formi artikla. Portal: polje i
kolona. Rok trajanja ostaje obavezan pri prijemu za artikle sa pracenjem roka.
Testovi: test_package_barcode.py.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015juQkhMLCFcM7xgeZe5c3A
</commit_message>
<xml_diff>
--- a/.claude/DOCS/primer-uvoz-artikala.xlsx
+++ b/.claude/DOCS/primer-uvoz-artikala.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Artikli" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Artikli" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -414,17 +414,19 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H9"/>
+  <dimension ref="A1:J9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="32" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
     <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -468,6 +470,16 @@
           <t>Stanje (komada)</t>
         </is>
       </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>Prati rok (da/ne)</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>Barkod kutije</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -500,6 +512,16 @@
       <c r="H2" t="n">
         <v>240</v>
       </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="J2" s="1" t="inlineStr">
+        <is>
+          <t>8601000100011</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -517,10 +539,8 @@
           <t>Bambi</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>189.9</t>
-        </is>
+      <c r="D3" t="n">
+        <v>189.9</v>
       </c>
       <c r="E3" t="n">
         <v>20</v>
@@ -533,6 +553,16 @@
       </c>
       <c r="H3" t="n">
         <v>120</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="J3" s="1" t="inlineStr">
+        <is>
+          <t>8601000100028</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -562,6 +592,12 @@
       <c r="H4" t="n">
         <v>0</v>
       </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="J4" s="1" t="n"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -596,6 +632,16 @@
       <c r="H5" t="n">
         <v>360</v>
       </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="J5" s="1" t="inlineStr">
+        <is>
+          <t>8601000100042</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -628,6 +674,12 @@
       <c r="H6" t="n">
         <v>300</v>
       </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>da</t>
+        </is>
+      </c>
+      <c r="J6" s="1" t="n"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -645,10 +697,8 @@
           <t>Dijamant</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>259</t>
-        </is>
+      <c r="D7" t="n">
+        <v>259</v>
       </c>
       <c r="E7" t="n">
         <v>20</v>
@@ -662,6 +712,12 @@
       <c r="H7" t="n">
         <v>180</v>
       </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="J7" s="1" t="n"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -679,8 +735,10 @@
           <t>Mlin</t>
         </is>
       </c>
-      <c r="D8" t="n">
-        <v>79.90000000000001</v>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>79,9</t>
+        </is>
       </c>
       <c r="E8" t="n">
         <v>10</v>
@@ -694,6 +752,12 @@
       <c r="H8" t="n">
         <v>500</v>
       </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="J8" s="1" t="n"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -711,10 +775,8 @@
           <t>Strauss</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>299</t>
-        </is>
+      <c r="D9" t="n">
+        <v>299</v>
       </c>
       <c r="E9" t="n">
         <v>20</v>
@@ -725,6 +787,12 @@
       <c r="G9" t="n">
         <v>48</v>
       </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="J9" s="1" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Jedinice mere: kolona Jedinica mere u Excel uvozu artikala (stanje u izabranoj jedinici)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015juQkhMLCFcM7xgeZe5c3A
</commit_message>
<xml_diff>
--- a/.claude/DOCS/primer-uvoz-artikala.xlsx
+++ b/.claude/DOCS/primer-uvoz-artikala.xlsx
@@ -414,7 +414,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J9"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -424,9 +424,10 @@
     <col width="8" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="30" customWidth="1" min="7" max="7"/>
-    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
     <col width="18" customWidth="1" min="9" max="9"/>
     <col width="18" customWidth="1" min="10" max="10"/>
+    <col width="16" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -467,7 +468,7 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
-          <t>Stanje (komada)</t>
+          <t>Stanje (u jedinici mere)</t>
         </is>
       </c>
       <c r="I1" t="inlineStr">
@@ -478,6 +479,11 @@
       <c r="J1" t="inlineStr">
         <is>
           <t>Barkod kutije</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>Jedinica mere</t>
         </is>
       </c>
     </row>
@@ -522,6 +528,11 @@
           <t>8601000100011</t>
         </is>
       </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -564,6 +575,11 @@
           <t>8601000100028</t>
         </is>
       </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -598,6 +614,11 @@
         </is>
       </c>
       <c r="J4" s="1" t="n"/>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -642,6 +663,11 @@
           <t>8601000100042</t>
         </is>
       </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -680,6 +706,11 @@
         </is>
       </c>
       <c r="J6" s="1" t="n"/>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -718,6 +749,11 @@
         </is>
       </c>
       <c r="J7" s="1" t="n"/>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -758,6 +794,11 @@
         </is>
       </c>
       <c r="J8" s="1" t="n"/>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -793,6 +834,56 @@
         </is>
       </c>
       <c r="J9" s="1" t="n"/>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>kom</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Sir kačkavalj (po kg)</t>
+        </is>
+      </c>
+      <c r="B10" s="1" t="inlineStr">
+        <is>
+          <t>8601000000094</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>Mlekara</t>
+        </is>
+      </c>
+      <c r="D10" t="n">
+        <v>1100</v>
+      </c>
+      <c r="E10" t="n">
+        <v>10</v>
+      </c>
+      <c r="F10" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>25,5</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>ne</t>
+        </is>
+      </c>
+      <c r="J10" s="1" t="n"/>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>kg</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>